<commit_message>
fix: exist and mail
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RPA02\Documents\UiPath\REF_RPA\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEEC3FCF-6ACC-4626-88B2-398C1F73252B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8537229-A76D-40FE-B926-31A521AB299A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -258,7 +258,7 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>C:\Users\RPA02\Desktop\release_v1.0.85</t>
+    <t>C:\Users\RPA02\Desktop\release_v1.0.86</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>

</xml_diff>

<commit_message>
fix: ui & add mail
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RPA02\Documents\UiPath\REF_RPA\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D92ABC09-93D8-46D9-A141-AAF5554668E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCD3F35C-EA0D-4C6C-B88B-F44145CD5FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="73">
   <si>
     <t>Name</t>
   </si>
@@ -260,13 +260,29 @@
   <si>
     <t>C:\Users\RPA02\Desktop\release_v1.0.86</t>
     <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <t>DB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>생명</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -302,6 +318,13 @@
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2891,7 +2914,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77CF0077-C10E-4F26-8041-D603A9E1E372}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
@@ -2934,133 +2957,122 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B13" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="C13" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B14" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C14" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>65</v>
-      </c>
-      <c r="B15" t="s">
-        <v>66</v>
-      </c>
-      <c r="C15" t="s">
         <v>66</v>
       </c>
     </row>
@@ -3124,15 +3136,15 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" ht="17.399999999999999">
       <c r="A5" t="s">
         <v>45</v>
       </c>
       <c r="B5" t="s">
         <v>46</v>
       </c>
-      <c r="C5" t="s">
-        <v>46</v>
+      <c r="C5" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:3">

</xml_diff>

<commit_message>
fix: email to assets
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RPA02\Documents\UiPath\REF_RPA\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RPA02\Documents\UiPath\RPA\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCD3F35C-EA0D-4C6C-B88B-F44145CD5FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19CFEAE1-2883-4AFA-BD47-9B90B8CE6888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: program to send params
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RPA02\Documents\UiPath\RPA\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DE24ADC-3DCF-4794-8018-98C23D47E640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2573ED8-D044-427C-8141-D120D45AF638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -274,7 +274,7 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>C:\Users\RPA02\Desktop\release_v1.0.88</t>
+    <t>C:\Users\RPA02\Desktop\release_v1.0.90</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>

</xml_diff>

<commit_message>
fix: upload hardware event
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RPA02\Documents\UiPath\RPA\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{353F0CF0-89AB-4E82-9795-4E7DAD29B56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07672A24-5E45-4EF5-A09E-FAEA51288D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="73">
   <si>
     <t>Name</t>
   </si>
@@ -2914,7 +2914,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77CF0077-C10E-4F26-8041-D603A9E1E372}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
@@ -2990,100 +2990,89 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B13" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="C13" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B14" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C14" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>65</v>
-      </c>
-      <c r="B15" t="s">
-        <v>66</v>
-      </c>
-      <c r="C15" t="s">
         <v>66</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: ltg & ssf upload
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RPA02\Documents\UiPath\RPA\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07672A24-5E45-4EF5-A09E-FAEA51288D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E12D981A-F5DA-46D0-854A-8A1423BF3D8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="73">
   <si>
     <t>Name</t>
   </si>
@@ -2914,7 +2914,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77CF0077-C10E-4F26-8041-D603A9E1E372}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
@@ -2990,89 +2990,100 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="B11" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="C11" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B13" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
         <v>65</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
         <v>66</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C15" t="s">
         <v>66</v>
       </c>
     </row>

</xml_diff>